<commit_message>
Estudo 11: mesma revisão de linguagem na nota técnica e na planilha
Espelha na planilha e no PDF as mudanças feitas na página: troca "bolo"
por "arrecadação"/"receita total", explica em linguagem simples o que
significa a arrecadação crescer na mesma proporção do PIB (em vez de só
citar "elasticidade"), e limpa travessões e menções a outros estudos que
tinham ficado de fora da revisão anterior (a planilha não tinha sido
tocada naquela passada).
</commit_message>
<xml_diff>
--- a/materiais/ibs-projecao-nacional-memoria-calculo.xlsx
+++ b/materiais/ibs-projecao-nacional-memoria-calculo.xlsx
@@ -521,14 +521,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Estudo 11 — IBS total do Brasil, 2029-2033</t>
+          <t>Estudo 11: IBS total do Brasil, 2029-2033</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Série histórica (2015-2025) e projeção com PIB e inflação oficiais — memória de cálculo</t>
+          <t>Série histórica (2015-2025) e projeção com PIB e inflação oficiais, memória de cálculo</t>
         </is>
       </c>
     </row>
@@ -563,12 +563,12 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Bolo total em 2033 (ICMS+ISS+IBS)</t>
+          <t>Arrecadação total em 2033 (ICMS+ISS+IBS)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>R$ 1,608.6 bi (8.08% do PIB — mesma proporção de 2025, por premissa)</t>
+          <t>R$ 1,608.6 bi (8.08% do PIB, a mesma proporção de 2025, por premissa)</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Razão ICMS+ISS/PIB constante no nível de 2025 a partir de 2026 (elasticidade-PIB unitária) — mesma premissa de neutralidade de receita do art. 130 ADCT usada nos Estudos 06 e 09 do site.</t>
+          <t>A arrecadação de ICMS e ISS, como proporção do PIB (a carga tributária), é mantida constante no nível de 2025 a partir de 2026: ela cresce sempre no mesmo ritmo da economia, nem mais nem menos rápido. É o próprio desenho legal da transição para o IBS (art. 130, caput e §3º, IV, do ADCT: o Senado fixa a alíquota de referência do IBS para manter a Receita-Base dos Entes Subnacionais como proporção do PIB).</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>IFI — Instituição Fiscal Independente (Senado Federal), Relatório de Acompanhamento Fiscal (RAF) nº 107, 18/dez/2025: PIB real 2,2% a.a. (2027-2035), IPCA convergindo a 3,0% (centro da meta contínua).</t>
+          <t>IFI, Instituição Fiscal Independente (Senado Federal), Relatório de Acompanhamento Fiscal (RAF) nº 107, 18/dez/2025: PIB real 2,2% a.a. (2027-2035), IPCA convergindo a 3,0% (centro da meta contínua).</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SICONFI/STN — RREO Anexo 3 (2015-2018) e DCA Anexo I-C (2019-2025).</t>
+          <t>SICONFI/STN, RREO Anexo 3 (2015-2018) e DCA Anexo I-C (2019-2025).</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SICONFI/STN — DCA Anexo I-C, todos os municípios brasileiros (2015-2025).</t>
+          <t>SICONFI/STN, DCA Anexo I-C, todos os municípios brasileiros (2015-2025).</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Idêntico ao usado no Estudo 06 (Projeção ICMS/IBS por Estado, 2029-2033).</t>
+          <t>Fração remanescente de ICMS/ISS (f_a) e fração já convertida em IBS (s_a=1-f_a) a cada ano da transição, conforme ADCT arts. 128 e 131.</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Aba 'Série histórica': dados de entrada SICONFI 2015-2025. Aba 'Premissas macro': dados de entrada Focus/IFI 2026-2033. Aba 'PIB projetado': fórmulas que compõem o PIB nominal ano a ano. Aba 'Projeção IBS': fórmulas que aplicam a razão bolo/PIB e o cronograma ADCT — mude qualquer premissa nas abas de entrada (em azul) e a projeção recalcula.</t>
+          <t>Aba 'Série histórica': dados de entrada SICONFI 2015-2025. Aba 'Premissas macro': dados de entrada Focus/IFI 2026-2033. Aba 'PIB projetado': fórmulas que compõem o PIB nominal ano a ano. Aba 'Projeção IBS': fórmulas que aplicam a carga tributária constante e o cronograma ADCT. Mude qualquer premissa nas abas de entrada (em azul) e a projeção recalcula.</t>
         </is>
       </c>
     </row>
@@ -742,14 +742,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ICMS + ISS, Brasil — série histórica 2015-2025</t>
+          <t>ICMS + ISS, Brasil: série histórica 2015-2025</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dados de entrada (células em azul) — SICONFI/STN</t>
+          <t>Dados de entrada (células em azul), SICONFI/STN</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dados de entrada (células em azul) — Boletim Focus (BCB) e IFI (RAF 107)</t>
+          <t>Dados de entrada (células em azul), Boletim Focus (BCB) e IFI (RAF 107)</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
     <row r="14" ht="55" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>2026-2030: mediana do Boletim Focus (BCB), consultada via API do Sistema de Expectativas de Mercado. 2031-2033: fora do horizonte do Focus (~5 anos); usa-se a projeção da IFI (RAF 107, 18/dez/2025), constante nos três anos por simplificação — a IFI projeta uma taxa média para 2027-2035, não ano a ano.</t>
+          <t>2026-2030: mediana do Boletim Focus (BCB), consultada via API do Sistema de Expectativas de Mercado. 2031-2033: fora do horizonte do Focus (~5 anos); usa-se a projeção da IFI (RAF 107, 18/dez/2025), constante nos três anos por simplificação, já que a IFI projeta uma taxa média para 2027-2035, não ano a ano.</t>
         </is>
       </c>
     </row>
@@ -1534,14 +1534,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fórmulas: Bolo(t) = (Bolo2025/PIB2025) × PIB(t); ICMS+ISS residual = Bolo × fa; IBS bruto = Bolo × sa</t>
+          <t>Fórmulas: Receita(t) = (Receita2025/PIB2025) × PIB(t); ICMS+ISS residual = Receita × fa; IBS bruto = Receita × sa</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Razão bolo/PIB em 2025 (base):</t>
+          <t>Carga tributária (arrecadação/PIB) em 2025, base da projeção:</t>
         </is>
       </c>
       <c r="B4" s="16">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Bolo projetado (R$)</t>
+          <t>Receita projetada (R$)</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Bolo / PIB</t>
+          <t>Carga tributária (% PIB)</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
     <row r="13" ht="55" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>f_a (fração remanescente de ICMS+ISS) e s_a=1-f_a (fração já convertida em IBS) seguem o cronograma da transição constitucional (ADCT arts. 128 e 131, LC 227/2026), idêntico ao usado no Estudo 06 (Projeção ICMS/IBS por Estado). "IBS bruto" não desconta a taxa do CGIBS nem a retenção do Seguro-Receita (ADCT art. 132), que incidem sobre a parcela distribuída aos entes pelo critério destino — não sobre o total nacional.</t>
+          <t>f_a (fração remanescente de ICMS+ISS) e s_a=1-f_a (fração já convertida em IBS) seguem o cronograma da transição constitucional (ADCT arts. 128 e 131, LC 227/2026). "IBS bruto" não desconta a taxa do CGIBS nem a retenção do Seguro-Receita (ADCT art. 132), que incidem sobre a parcela distribuída aos entes pelo critério destino, não sobre o total nacional.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Estudo 11: explica por que o Teto de Referência não muda a projeção
Detalha o mecanismo do art. 130, §4º e §5º, do ADCT: compara a média
2029-2033 de CBS+Imposto Seletivo+IBS com a média 2012-2021 de
IPI+ICMS+ISS+PIS/Cofins+IOF-seguros. Explicita os dois motivos por que
isso não exige recalcular nada: (i) mesmo se ultrapassado, a redução da
alíquota só vale a partir de 2035, fora da janela 2029-2033 projetada
aqui; (ii) o teto soma o lado federal (fora do escopo deste estudo) ao
subnacional, então simulá-lo exigiria dados que este site não coleta.

Sem mudança nos números: só a explicação metodológica, replicada na
página, na nota técnica e na planilha.
</commit_message>
<xml_diff>
--- a/materiais/ibs-projecao-nacional-memoria-calculo.xlsx
+++ b/materiais/ibs-projecao-nacional-memoria-calculo.xlsx
@@ -101,7 +101,7 @@
     <t xml:space="preserve">Gerado em</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-31</t>
+    <t xml:space="preserve">2026-08-01</t>
   </si>
   <si>
     <t xml:space="preserve">Página do estudo</t>
@@ -212,7 +212,7 @@
     <t xml:space="preserve">Média 2024-2026 (usada na projeção)</t>
   </si>
   <si>
-    <t xml:space="preserve">O Teto de Referência do art. 130, §4º e §5º, do ADCT usa outro período (média 2012-2021) como salvaguarda, não como base de cálculo ano a ano da alíquota; não é usado nesta planilha.</t>
+    <t xml:space="preserve">O Teto de Referência (ADCT art. 130, §4º e §5º) compara a média 2029-2033 de CBS+Imposto Seletivo+IBS com a média 2012-2021 de IPI+ICMS+ISS+PIS/Cofins+IOF-seguros. Não altera os valores desta planilha: mesmo se ultrapassado, a redução só vale a partir de 2035 (fora desta projeção), e exige dados federais fora do escopo deste estudo (só ICMS/ISS/IBS).</t>
   </si>
   <si>
     <t xml:space="preserve">f_a (ICMS+ISS residual)</t>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="E9" s="14"/>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
         <v>62</v>
       </c>

</xml_diff>